<commit_message>
update the ranges of the time-series parameters and the initial values of environmental variables
</commit_message>
<xml_diff>
--- a/input_params_range.xlsx
+++ b/input_params_range.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiawei/Documents/Work/2024- loessPSM/paleosolCO2_CLP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{286E12A0-4F4F-0B48-9AF6-4D8F858E620F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D9ACF27-94A7-5F45-8E95-D87855F64904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12560" yWindow="3520" windowWidth="28040" windowHeight="17440" xr2:uid="{C89A10F1-C584-8C4D-85A3-B57BD1FEEBA8}"/>
+    <workbookView xWindow="9720" yWindow="3500" windowWidth="28040" windowHeight="17440" xr2:uid="{C89A10F1-C584-8C4D-85A3-B57BD1FEEBA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -95,9 +95,6 @@
     <t>0-20</t>
   </si>
   <si>
-    <t>7-13</t>
-  </si>
-  <si>
     <t>PCQ_to</t>
   </si>
   <si>
@@ -131,12 +128,6 @@
     <t>Modern observations from the CLP</t>
   </si>
   <si>
-    <t>100-400</t>
-  </si>
-  <si>
-    <t>Yang et al., 2015, PNAS</t>
-  </si>
-  <si>
     <t>PCQ_pf</t>
   </si>
   <si>
@@ -146,19 +137,28 @@
     <t>0-1</t>
   </si>
   <si>
-    <t>0.4-0.55</t>
-  </si>
-  <si>
     <t>tsc</t>
   </si>
   <si>
     <t>timing of pedogenic carbonate formation</t>
   </si>
   <si>
-    <t>0.4-0.5</t>
-  </si>
-  <si>
-    <t>Da et al., 2023, QSR</t>
+    <t>10-17</t>
+  </si>
+  <si>
+    <t>200-750</t>
+  </si>
+  <si>
+    <t>0.26-0.55</t>
+  </si>
+  <si>
+    <t>Meng et al., 2018; Yang et al., 2015</t>
+  </si>
+  <si>
+    <t>Da et al., 2023; Modern observations</t>
+  </si>
+  <si>
+    <t>0.34-0.55</t>
   </si>
 </sst>
 </file>
@@ -568,7 +568,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -588,7 +588,7 @@
         <v>9</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -608,7 +608,7 @@
         <v>14</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -625,18 +625,18 @@
         <v>18</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>17</v>
@@ -645,70 +645,70 @@
         <v>18</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>25</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>